<commit_message>
Uygulama arayuzunu ve oyun ozelliklerini guncelle
</commit_message>
<xml_diff>
--- a/flutter_application_1/101_Okey_Seviye_ve_Ekonomi_Kurallari.xlsx
+++ b/flutter_application_1/101_Okey_Seviye_ve_Ekonomi_Kurallari.xlsx
@@ -5,18 +5,19 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\evren\OneDrive\Masaüstü\101okey\flutter_application_1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gokde\OneDrive\Desktop\101\101\flutter_application_1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7B3732A8-E9A3-4205-B51C-06214621CB20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05EBE5C9-F93F-4C2C-8F50-0CFF057C2DEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="384" yWindow="384" windowWidth="17280" windowHeight="8880" xr2:uid="{DE1AD867-BDFB-49D0-A2A8-64F4CF1669D1}"/>
+    <workbookView xWindow="-28920" yWindow="-975" windowWidth="29040" windowHeight="15720" xr2:uid="{DE1AD867-BDFB-49D0-A2A8-64F4CF1669D1}"/>
   </bookViews>
   <sheets>
-    <sheet name="Genel Kurallar" sheetId="4" r:id="rId1"/>
-    <sheet name="Oyun XP Kazanımları" sheetId="3" r:id="rId2"/>
-    <sheet name="Seviye Tablosu" sheetId="2" r:id="rId3"/>
-    <sheet name="Altın Ekonomisi" sheetId="1" r:id="rId4"/>
+    <sheet name="Masa Seviye Kilitleri" sheetId="5" r:id="rId1"/>
+    <sheet name="Genel Kurallar" sheetId="4" r:id="rId2"/>
+    <sheet name="Oyun XP Kazanımları" sheetId="3" r:id="rId3"/>
+    <sheet name="Seviye Tablosu" sheetId="2" r:id="rId4"/>
+    <sheet name="Altın Ekonomisi" sheetId="1" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="104">
   <si>
     <t>Kural</t>
   </si>
@@ -53,9 +54,6 @@
     <t>Başlangıç seviyesi</t>
   </si>
   <si>
-    <t>Mevcut test profili: Seviye 9 - Learner. Yeni oyuncu için önerilen: Seviye 1 - Beginner.</t>
-  </si>
-  <si>
     <t>Seviye atlama</t>
   </si>
   <si>
@@ -83,9 +81,6 @@
     <t>Örnek</t>
   </si>
   <si>
-    <t>Seviye 9'da 40/50 XP bulunan oyuncu 30 XP kazanırsa Seviye 10 ve 20/50 XP olur.</t>
-  </si>
-  <si>
     <t>Oyun Türü</t>
   </si>
   <si>
@@ -239,9 +234,6 @@
     <t>Champion</t>
   </si>
   <si>
-    <t>95-99</t>
-  </si>
-  <si>
     <t>Grandmaster</t>
   </si>
   <si>
@@ -291,13 +283,85 @@
   </si>
   <si>
     <t>Aşama ilerledikçe ödül artar</t>
+  </si>
+  <si>
+    <t>Yeni oyuncu Seviye 0 - Beginner ve 0/30 XP ile başlar.</t>
+  </si>
+  <si>
+    <t>Seviye 3'te 20/30 XP bulunan oyuncu 30 XP kazanırsa Seviye 4 ve 20/50 XP olur.</t>
+  </si>
+  <si>
+    <t>0-2</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>5-7</t>
+  </si>
+  <si>
+    <t>8-9</t>
+  </si>
+  <si>
+    <t>10-12</t>
+  </si>
+  <si>
+    <t>13-14</t>
+  </si>
+  <si>
+    <t>95-98</t>
+  </si>
+  <si>
+    <t>99</t>
+  </si>
+  <si>
+    <t>MAX</t>
+  </si>
+  <si>
+    <t>Masa</t>
+  </si>
+  <si>
+    <t>Gerekli Seviye</t>
+  </si>
+  <si>
+    <t>Giriş Ücreti</t>
+  </si>
+  <si>
+    <t>Durum</t>
+  </si>
+  <si>
+    <t>Başlangıç</t>
+  </si>
+  <si>
+    <t>Başlangıçta açık</t>
+  </si>
+  <si>
+    <t>Standart</t>
+  </si>
+  <si>
+    <t>5. seviyede açılır</t>
+  </si>
+  <si>
+    <t>VIP</t>
+  </si>
+  <si>
+    <t>15. seviyede açılır</t>
+  </si>
+  <si>
+    <t>Elit</t>
+  </si>
+  <si>
+    <t>25. seviyede açılır</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -330,6 +394,14 @@
       <charset val="162"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -345,7 +417,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -368,22 +440,39 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="16" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -402,7 +491,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Teması">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -717,6 +806,92 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFCCF1CE-1A74-497E-86FF-8788F2D9FBB4}">
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="B2" s="6">
+        <v>0</v>
+      </c>
+      <c r="C2" s="6">
+        <v>500</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="B3" s="6">
+        <v>5</v>
+      </c>
+      <c r="C3" s="6">
+        <v>1000</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="B4" s="6">
+        <v>15</v>
+      </c>
+      <c r="C4" s="6">
+        <v>5000</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="B5" s="6">
+        <v>25</v>
+      </c>
+      <c r="C5" s="6">
+        <v>10000</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>103</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4001ADE0-0EBC-4C07-8D6A-4A34DD13E9FC}">
   <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -738,47 +913,47 @@
         <v>2</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>3</v>
+        <v>80</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>4</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>8</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>10</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>13</v>
+        <v>81</v>
       </c>
     </row>
   </sheetData>
@@ -786,7 +961,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5530FC9-11B2-490C-80F1-040962266B08}">
   <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -797,27 +972,27 @@
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="F1" s="2" t="s">
         <v>17</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B2" s="3">
         <v>30</v>
@@ -837,7 +1012,7 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B3" s="3">
         <v>30</v>
@@ -857,7 +1032,7 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B4" s="3">
         <v>35</v>
@@ -877,7 +1052,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B5" s="3">
         <v>50</v>
@@ -897,270 +1072,15 @@
     </row>
     <row r="6" spans="1:6" ht="72" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C169857D-6A2D-4D81-99F3-8B60C098C41D}">
-  <dimension ref="A1:C22"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="3" width="22.77734375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="4">
-        <v>46024</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="C2" s="3">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="4">
-        <v>46085</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="C3" s="3">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A4" s="4">
-        <v>46151</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="C4" s="3">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="4">
-        <v>46309</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="C5" s="3">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A6" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="C6" s="3">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="C7" s="3">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A8" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="C8" s="3">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A9" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="C9" s="3">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A10" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="C10" s="3">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A11" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="C11" s="3">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A12" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="C12" s="3">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="C13" s="3">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A14" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="C14" s="3">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="C15" s="3">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="C16" s="3">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="C17" s="3">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="C18" s="3">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="C19" s="3">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="C20" s="3">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="C21" s="3">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A22" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="C22" s="3">
-        <v>150</v>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1168,6 +1088,307 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C169857D-6A2D-4D81-99F3-8B60C098C41D}">
+  <dimension ref="A1:C26"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C2" s="3">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C3" s="3">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" s="3">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" s="3">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C8" s="3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" s="3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C10" s="3">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C11" s="3">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C12" s="3">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C13" s="3">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C14" s="3">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C15" s="3">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="C16" s="3">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C17" s="3">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="C18" s="3">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C19" s="3">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C20" s="3">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C21" s="3">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C22" s="3">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C23" s="3">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C24" s="3">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C25" s="3">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>91</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E80A4773-6FB8-4EB3-BB73-2423A6DD7072}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1179,10 +1400,10 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>1</v>
@@ -1190,68 +1411,68 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B2" s="3">
         <v>25600</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B3" s="3">
         <v>150</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B4" s="3">
         <v>300</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
101 Okey mevcut oyun, arayuz ve ogretici guncellemelerini kaydet
</commit_message>
<xml_diff>
--- a/flutter_application_1/101_Okey_Seviye_ve_Ekonomi_Kurallari.xlsx
+++ b/flutter_application_1/101_Okey_Seviye_ve_Ekonomi_Kurallari.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gokde\OneDrive\Desktop\101\101\flutter_application_1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d4b3de4e1ba46f8a/Desktop/101/101/flutter_application_1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05EBE5C9-F93F-4C2C-8F50-0CFF057C2DEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="17" documentId="13_ncr:1_{05EBE5C9-F93F-4C2C-8F50-0CFF057C2DEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FB616B7D-4DCE-44E9-A756-7615BE57E678}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-975" windowWidth="29040" windowHeight="15720" xr2:uid="{DE1AD867-BDFB-49D0-A2A8-64F4CF1669D1}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{DE1AD867-BDFB-49D0-A2A8-64F4CF1669D1}"/>
   </bookViews>
   <sheets>
     <sheet name="Masa Seviye Kilitleri" sheetId="5" r:id="rId1"/>
@@ -19,21 +19,10 @@
     <sheet name="Seviye Tablosu" sheetId="2" r:id="rId4"/>
     <sheet name="Altın Ekonomisi" sheetId="1" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="2"/>
@@ -43,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="109">
   <si>
     <t>Kural</t>
   </si>
@@ -96,9 +85,6 @@
     <t>Eli Bitirme</t>
   </si>
   <si>
-    <t>Azami XP</t>
-  </si>
-  <si>
     <t>Hemen Oyna</t>
   </si>
   <si>
@@ -246,9 +232,6 @@
     <t>Başlangıç bakiyesi</t>
   </si>
   <si>
-    <t>Mevcut varsayılan hesap bakiyesi</t>
-  </si>
-  <si>
     <t>Hemen Oyna galibiyeti</t>
   </si>
   <si>
@@ -288,9 +271,6 @@
     <t>Yeni oyuncu Seviye 0 - Beginner ve 0/30 XP ile başlar.</t>
   </si>
   <si>
-    <t>Seviye 3'te 20/30 XP bulunan oyuncu 30 XP kazanırsa Seviye 4 ve 20/50 XP olur.</t>
-  </si>
-  <si>
     <t>0-2</t>
   </si>
   <si>
@@ -355,6 +335,30 @@
   </si>
   <si>
     <t>25. seviyede açılır</t>
+  </si>
+  <si>
+    <t>Seviye 3'te 20/50 XP bulunan oyuncu 40 XP kazanırsa Seviye 4 ve 10/50 XP olur.</t>
+  </si>
+  <si>
+    <t>1. Tur Azami XP</t>
+  </si>
+  <si>
+    <t>Tur galibiyeti bonusu</t>
+  </si>
+  <si>
+    <t>+10 x (tur no - 1)</t>
+  </si>
+  <si>
+    <t>En çok +200 XP</t>
+  </si>
+  <si>
+    <t>Uygulamadaki varsayılan ve ilk geçiş bakiyesi</t>
+  </si>
+  <si>
+    <t>+50 x (tur no - 1)</t>
+  </si>
+  <si>
+    <t>Kazanana 2. turdan itibaren verilir; en çok +1.000 altın</t>
   </si>
 </sst>
 </file>
@@ -403,7 +407,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -413,6 +417,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -459,7 +469,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -473,6 +483,10 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -818,21 +832,21 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="D1" s="5" t="s">
         <v>92</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="B2" s="6">
         <v>0</v>
@@ -841,12 +855,12 @@
         <v>500</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="B3" s="6">
         <v>5</v>
@@ -855,12 +869,12 @@
         <v>1000</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B4" s="6">
         <v>15</v>
@@ -869,12 +883,12 @@
         <v>5000</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B5" s="6">
         <v>25</v>
@@ -883,7 +897,7 @@
         <v>10000</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -913,7 +927,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -953,7 +967,7 @@
         <v>11</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>81</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>
@@ -963,7 +977,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5530FC9-11B2-490C-80F1-040962266B08}">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24.77734375" customWidth="1"/>
@@ -987,12 +1001,12 @@
         <v>16</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>17</v>
+        <v>102</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B2" s="3">
         <v>30</v>
@@ -1012,7 +1026,7 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B3" s="3">
         <v>30</v>
@@ -1032,7 +1046,7 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B4" s="3">
         <v>35</v>
@@ -1052,7 +1066,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B5" s="3">
         <v>50</v>
@@ -1070,17 +1084,31 @@
         <v>150</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="72" x14ac:dyDescent="0.3">
-      <c r="A6" s="3" t="s">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="C6" s="7"/>
+      <c r="D6" s="7"/>
+      <c r="E6" s="7"/>
+      <c r="F6" s="7" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="72" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B6" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1099,21 +1127,21 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>25</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C2" s="3">
         <v>30</v>
@@ -1121,21 +1149,21 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C3" s="3">
-        <v>30</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C4" s="3">
         <v>50</v>
@@ -1143,21 +1171,21 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C5" s="3">
-        <v>50</v>
+        <v>65</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C6" s="3">
         <v>75</v>
@@ -1165,10 +1193,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C7" s="3">
         <v>75</v>
@@ -1176,10 +1204,10 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C8" s="3">
         <v>100</v>
@@ -1187,10 +1215,10 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>31</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>32</v>
       </c>
       <c r="C9" s="3">
         <v>100</v>
@@ -1198,10 +1226,10 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" s="3" t="s">
         <v>33</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>34</v>
       </c>
       <c r="C10" s="3">
         <v>130</v>
@@ -1209,10 +1237,10 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B11" s="3" t="s">
         <v>35</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>36</v>
       </c>
       <c r="C11" s="3">
         <v>130</v>
@@ -1220,10 +1248,10 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B12" s="3" t="s">
         <v>37</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>38</v>
       </c>
       <c r="C12" s="3">
         <v>170</v>
@@ -1231,10 +1259,10 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B13" s="3" t="s">
         <v>39</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>40</v>
       </c>
       <c r="C13" s="3">
         <v>170</v>
@@ -1242,10 +1270,10 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="B14" s="3" t="s">
         <v>41</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>42</v>
       </c>
       <c r="C14" s="3">
         <v>170</v>
@@ -1253,10 +1281,10 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="B15" s="3" t="s">
         <v>43</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>44</v>
       </c>
       <c r="C15" s="3">
         <v>220</v>
@@ -1264,10 +1292,10 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B16" s="3" t="s">
         <v>45</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>46</v>
       </c>
       <c r="C16" s="3">
         <v>220</v>
@@ -1275,10 +1303,10 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="B17" s="3" t="s">
         <v>47</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>48</v>
       </c>
       <c r="C17" s="3">
         <v>220</v>
@@ -1286,10 +1314,10 @@
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B18" s="3" t="s">
         <v>49</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>50</v>
       </c>
       <c r="C18" s="3">
         <v>280</v>
@@ -1297,10 +1325,10 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B19" s="3" t="s">
         <v>51</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>52</v>
       </c>
       <c r="C19" s="3">
         <v>280</v>
@@ -1308,10 +1336,10 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B20" s="3" t="s">
         <v>53</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>54</v>
       </c>
       <c r="C20" s="3">
         <v>280</v>
@@ -1319,10 +1347,10 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B21" s="3" t="s">
         <v>55</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>56</v>
       </c>
       <c r="C21" s="3">
         <v>350</v>
@@ -1330,10 +1358,10 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="B22" s="3" t="s">
         <v>57</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>58</v>
       </c>
       <c r="C22" s="3">
         <v>350</v>
@@ -1341,10 +1369,10 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="B23" s="3" t="s">
         <v>59</v>
-      </c>
-      <c r="B23" s="3" t="s">
-        <v>60</v>
       </c>
       <c r="C23" s="3">
         <v>350</v>
@@ -1352,10 +1380,10 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B24" s="3" t="s">
         <v>61</v>
-      </c>
-      <c r="B24" s="3" t="s">
-        <v>62</v>
       </c>
       <c r="C24" s="3">
         <v>450</v>
@@ -1363,10 +1391,10 @@
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C25" s="3">
         <v>450</v>
@@ -1374,13 +1402,13 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
     </row>
   </sheetData>
@@ -1390,7 +1418,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E80A4773-6FB8-4EB3-BB73-2423A6DD7072}">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="28.77734375" customWidth="1"/>
@@ -1400,10 +1428,10 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>64</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>65</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>1</v>
@@ -1411,68 +1439,79 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B2" s="3">
-        <v>25600</v>
+        <v>100000</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>67</v>
+        <v>106</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B3" s="3">
         <v>150</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B4" s="3">
         <v>300</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>71</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>74</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="B7" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>79</v>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>108</v>
       </c>
     </row>
   </sheetData>

</xml_diff>